<commit_message>
Add lecture content, assets, and updated book output for publishing
Adds lecture 1-4 content updates, new image assets, introduction slides,
updated references, and rebuilt docs/ for GitHub Pages deployment.
Also updates .gitignore to exclude rendered lecture and readme HTML.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/heka22_lecture-overview-readings.xlsx
+++ b/heka22_lecture-overview-readings.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/research/teaching/heka22/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D4E1242C-DDD5-B94D-804A-38D08ABF28A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F11A87A-5341-E846-AE0F-90258491562A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{46322BC5-94F8-8B45-BA62-3179A18004EC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>

</xml_diff>

<commit_message>
WIP: Save lecture content, slides, assets, and references
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/heka22_lecture-overview-readings.xlsx
+++ b/heka22_lecture-overview-readings.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/research/teaching/heka22/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F11A87A-5341-E846-AE0F-90258491562A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1BCCB6E-08B7-7841-BF68-3B571BD8582D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{46322BC5-94F8-8B45-BA62-3179A18004EC}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="28">
   <si>
     <t>Lecture</t>
   </si>
@@ -118,12 +118,6 @@
       </rPr>
       <t xml:space="preserve"> 22 (2): 191–215. (24 s.)</t>
     </r>
-  </si>
-  <si>
-    <t>Foster, Clark &amp;
-York (2010). Hornborg
-(2006); Hornborg (2018); Spash
-(2017 kap. 4).</t>
   </si>
   <si>
     <t>Plural Perspectives: Eco Feminist Economics</t>
@@ -600,7 +594,7 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -617,7 +611,7 @@
     </row>
     <row r="2" spans="1:5" ht="51" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B2">
         <v>1</v>
@@ -634,7 +628,7 @@
     </row>
     <row r="3" spans="1:5" ht="85" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B3">
         <v>2</v>
@@ -651,7 +645,7 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B4">
         <v>3</v>
@@ -666,57 +660,55 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="68" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B5">
         <v>4</v>
       </c>
       <c r="C5" t="s">
-        <v>24</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>17</v>
-      </c>
+        <v>23</v>
+      </c>
+      <c r="D5" s="2"/>
     </row>
     <row r="7" spans="1:5" ht="255" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B7">
         <v>5</v>
       </c>
       <c r="C7" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>11</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="204" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B8">
         <v>6</v>
       </c>
       <c r="C8" t="s">
+        <v>17</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E8" s="2" t="s">
         <v>18</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B9">
         <v>7</v>
@@ -728,18 +720,18 @@
         <v>16</v>
       </c>
       <c r="E9" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="85" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B10">
         <v>8</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">

</xml_diff>